<commit_message>
Complete deep audit of 12_Quarters_Consolidated_Master.xlsx with zero missing values and trading-day-only verification
</commit_message>
<xml_diff>
--- a/Nifty50_Quarterly_Results_12_Quarters_Detailed_TradeLog_Master.xlsx
+++ b/Nifty50_Quarterly_Results_12_Quarters_Detailed_TradeLog_Master.xlsx
@@ -635,7 +635,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="116" customWidth="1" min="1" max="1"/>
     <col width="68" customWidth="1" min="2" max="2"/>
@@ -1766,7 +1766,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="179" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -5778,7 +5778,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="178" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -9790,7 +9790,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="179" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -13802,7 +13802,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="179" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -17814,7 +17814,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="179" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -21826,7 +21826,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="178" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -25838,7 +25838,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="178" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -29850,7 +29850,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="178" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -33862,7 +33862,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="178" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -37874,7 +37874,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="177" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -41886,7 +41886,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="178" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -45898,7 +45898,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:S60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="178" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>

</xml_diff>